<commit_message>
Update on the upper time window date
</commit_message>
<xml_diff>
--- a/ShinyApp/data/02_recent_adequacy.xlsx
+++ b/ShinyApp/data/02_recent_adequacy.xlsx
@@ -404,7 +404,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Butembo</t>
+          <t>Goma</t>
         </is>
       </c>
       <c r="B2">
@@ -416,10 +416,10 @@
         </is>
       </c>
       <c r="D2">
-        <v>-0.004525443073362112</v>
+        <v>-0.2165144085884094</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0.2228713780641556</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -435,7 +435,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Goma</t>
+          <t>Kalunguta</t>
         </is>
       </c>
       <c r="B3">
@@ -447,10 +447,10 @@
         </is>
       </c>
       <c r="D3">
-        <v>-0.2082830965518951</v>
+        <v>-0.04624922573566437</v>
       </c>
       <c r="E3">
-        <v>0.2428828179836273</v>
+        <v>0.8169167041778564</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -466,7 +466,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Kalunguta</t>
+          <t>Masereka</t>
         </is>
       </c>
       <c r="B4">
@@ -478,15 +478,21 @@
         </is>
       </c>
       <c r="D4">
-        <v>0.01388553995639086</v>
+        <v>0.210282951593399</v>
       </c>
       <c r="E4">
-        <v>0.9678783416748047</v>
+        <v>0.1997592449188232</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <v>0.3037569944044764</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -497,7 +503,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Masereka</t>
+          <t>Miti Murhesa</t>
         </is>
       </c>
       <c r="B5">
@@ -509,21 +515,15 @@
         </is>
       </c>
       <c r="D5">
-        <v>0.3085995316505432</v>
+        <v>-0.1292644441127777</v>
       </c>
       <c r="E5">
-        <v>0.06427383422851562</v>
+        <v>0.4387663602828979</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
-      </c>
-      <c r="G5">
-        <v>4</v>
-      </c>
-      <c r="H5">
-        <v>0.3104512843246658</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -534,7 +534,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Miti Murhesa</t>
+          <t>Viadana</t>
         </is>
       </c>
       <c r="B6">
@@ -546,15 +546,21 @@
         </is>
       </c>
       <c r="D6">
-        <v>-0.05703924596309662</v>
+        <v>0.2177862077951431</v>
       </c>
       <c r="E6">
-        <v>0.754699170589447</v>
+        <v>0.2296985387802124</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
+      </c>
+      <c r="G6">
+        <v>4</v>
+      </c>
+      <c r="H6">
+        <v>0.3037569944044764</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -565,11 +571,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Viadana</t>
+          <t>Gombari</t>
         </is>
       </c>
       <c r="B7">
-        <v>0</v>
+        <v>0.004761904761904762</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -577,21 +583,21 @@
         </is>
       </c>
       <c r="D7">
-        <v>0.2522251904010773</v>
+        <v>0.4658205211162567</v>
       </c>
       <c r="E7">
-        <v>0.1726109981536865</v>
+        <v>0.00719749927520752</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Increasing</t>
         </is>
       </c>
       <c r="G7">
         <v>4</v>
       </c>
       <c r="H7">
-        <v>0.3104512843246658</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -602,11 +608,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Makiso Kisangani</t>
+          <t>Tshopo</t>
         </is>
       </c>
       <c r="B8">
-        <v>0.009302713602184386</v>
+        <v>0.008620689655172414</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -614,10 +620,10 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.6199856996536255</v>
+        <v>0.4841409027576447</v>
       </c>
       <c r="E8">
-        <v>0.0001298189163208008</v>
+        <v>0.004570364952087402</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -628,7 +634,7 @@
         <v>4</v>
       </c>
       <c r="H8">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -643,7 +649,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>0.0101010101010101</v>
+        <v>0.009878193701723114</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -651,21 +657,21 @@
         </is>
       </c>
       <c r="D9">
-        <v>0.3136480152606964</v>
+        <v>0.4092455208301544</v>
       </c>
       <c r="E9">
-        <v>0.07140779495239258</v>
+        <v>0.01411116123199463</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Increasing</t>
         </is>
       </c>
       <c r="G9">
         <v>4</v>
       </c>
       <c r="H9">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -676,11 +682,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bafwasende</t>
+          <t>Makiso Kisangani</t>
         </is>
       </c>
       <c r="B10">
-        <v>0.01270878721859114</v>
+        <v>0.01383838383838384</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -688,10 +694,10 @@
         </is>
       </c>
       <c r="D10">
-        <v>0.4394488036632538</v>
+        <v>0.57316654920578</v>
       </c>
       <c r="E10">
-        <v>0.01008236408233643</v>
+        <v>0.0003368854522705078</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -702,7 +708,7 @@
         <v>4</v>
       </c>
       <c r="H10">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -713,11 +719,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ganga</t>
+          <t>Kabondo</t>
         </is>
       </c>
       <c r="B11">
-        <v>0.01636174326937379</v>
+        <v>0.01572327044025157</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -725,10 +731,10 @@
         </is>
       </c>
       <c r="D11">
-        <v>0.4220534563064575</v>
+        <v>0.5474497079849243</v>
       </c>
       <c r="E11">
-        <v>0.01992166042327881</v>
+        <v>0.000800013542175293</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -739,7 +745,7 @@
         <v>4</v>
       </c>
       <c r="H11">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -750,11 +756,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Rungu</t>
+          <t>Ganga</t>
         </is>
       </c>
       <c r="B12">
-        <v>0.01851851851851852</v>
+        <v>0.01631393298059965</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -762,10 +768,10 @@
         </is>
       </c>
       <c r="D12">
-        <v>0.5758761763572693</v>
+        <v>0.4845437407493591</v>
       </c>
       <c r="E12">
-        <v>0.0009148120880126953</v>
+        <v>0.005962848663330078</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -776,7 +782,7 @@
         <v>4</v>
       </c>
       <c r="H12">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -787,11 +793,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Wanierukula</t>
+          <t>Butembo</t>
         </is>
       </c>
       <c r="B13">
-        <v>0.02083333333333333</v>
+        <v>0.01783216783216783</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -799,21 +805,21 @@
         </is>
       </c>
       <c r="D13">
-        <v>0.5376822948455811</v>
+        <v>0.008116412907838821</v>
       </c>
       <c r="E13">
-        <v>0.001845359802246094</v>
+        <v>0.9793041944503784</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Increasing</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="G13">
         <v>4</v>
       </c>
       <c r="H13">
-        <v>0.3049138104028578</v>
+        <v>0.3058582486594755</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -824,11 +830,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gombari</t>
+          <t>Wanierukula</t>
         </is>
       </c>
       <c r="B14">
-        <v>0.02155202821869489</v>
+        <v>0.02083333333333334</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -836,10 +842,10 @@
         </is>
       </c>
       <c r="D14">
-        <v>0.4880623519420624</v>
+        <v>0.3696977496147156</v>
       </c>
       <c r="E14">
-        <v>0.006023645401000977</v>
+        <v>0.02988338470458984</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -850,7 +856,7 @@
         <v>4</v>
       </c>
       <c r="H14">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -861,11 +867,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tshopo</t>
+          <t>Adja</t>
         </is>
       </c>
       <c r="B15">
-        <v>0.02298850574712644</v>
+        <v>0.02380952380952381</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -873,10 +879,10 @@
         </is>
       </c>
       <c r="D15">
-        <v>0.5430247783660889</v>
+        <v>0.4639152884483337</v>
       </c>
       <c r="E15">
-        <v>0.001849889755249023</v>
+        <v>0.004813671112060547</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -887,7 +893,7 @@
         <v>4</v>
       </c>
       <c r="H15">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -898,11 +904,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Adja</t>
+          <t>Kambala</t>
         </is>
       </c>
       <c r="B16">
-        <v>0.02380952380952381</v>
+        <v>0.02718052738336714</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -910,10 +916,10 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.4449273645877838</v>
+        <v>0.390964537858963</v>
       </c>
       <c r="E16">
-        <v>0.009011268615722656</v>
+        <v>0.01713776588439941</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -924,7 +930,7 @@
         <v>4</v>
       </c>
       <c r="H16">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -935,11 +941,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Boga</t>
+          <t>Rungu</t>
         </is>
       </c>
       <c r="B17">
-        <v>0.02655228758169935</v>
+        <v>0.02740740740740741</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -947,21 +953,21 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.3125036358833313</v>
+        <v>0.6635317802429199</v>
       </c>
       <c r="E17">
-        <v>0.06418883800506592</v>
+        <v>6.771087646484375E-05</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Increasing</t>
         </is>
       </c>
       <c r="G17">
         <v>4</v>
       </c>
       <c r="H17">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -972,11 +978,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Rimba</t>
+          <t>Drodro</t>
         </is>
       </c>
       <c r="B18">
-        <v>0.02655691877620749</v>
+        <v>0.03472222222222222</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -984,10 +990,10 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.383610725402832</v>
+        <v>0.5603131055831909</v>
       </c>
       <c r="E18">
-        <v>0.01769483089447021</v>
+        <v>0.0002535581588745117</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -998,7 +1004,7 @@
         <v>4</v>
       </c>
       <c r="H18">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1009,11 +1015,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Kabondo</t>
+          <t>Lubunga</t>
         </is>
       </c>
       <c r="B19">
-        <v>0.02830188679245283</v>
+        <v>0.0425531914893617</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1021,10 +1027,10 @@
         </is>
       </c>
       <c r="D19">
-        <v>0.461042732000351</v>
+        <v>0.7224345207214355</v>
       </c>
       <c r="E19">
-        <v>0.006465554237365723</v>
+        <v>7.748603820800781E-06</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1035,7 +1041,7 @@
         <v>4</v>
       </c>
       <c r="H19">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1046,11 +1052,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Kambala</t>
+          <t>Ariwara</t>
         </is>
       </c>
       <c r="B20">
-        <v>0.0308316430020284</v>
+        <v>0.04444444444444445</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1058,10 +1064,10 @@
         </is>
       </c>
       <c r="D20">
-        <v>0.4170288443565369</v>
+        <v>0.562595546245575</v>
       </c>
       <c r="E20">
-        <v>0.01286780834197998</v>
+        <v>0.0003312826156616211</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1072,7 +1078,7 @@
         <v>4</v>
       </c>
       <c r="H20">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1083,11 +1089,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Lubero</t>
+          <t>Boga</t>
         </is>
       </c>
       <c r="B21">
-        <v>0.0407378046643993</v>
+        <v>0.04547803617571059</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1095,10 +1101,10 @@
         </is>
       </c>
       <c r="D21">
-        <v>0.6192871928215027</v>
+        <v>0.3697565793991089</v>
       </c>
       <c r="E21">
-        <v>0.0001165866851806641</v>
+        <v>0.02267980575561523</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1109,7 +1115,7 @@
         <v>4</v>
       </c>
       <c r="H21">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1120,11 +1126,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Lubunga</t>
+          <t>Bafwasende</t>
         </is>
       </c>
       <c r="B22">
-        <v>0.04964539007092199</v>
+        <v>0.05450636394908841</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1132,10 +1138,10 @@
         </is>
       </c>
       <c r="D22">
-        <v>0.734612762928009</v>
+        <v>0.5139064788818359</v>
       </c>
       <c r="E22">
-        <v>1.013278961181641E-05</v>
+        <v>0.001737356185913086</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1146,7 +1152,7 @@
         <v>4</v>
       </c>
       <c r="H22">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1157,11 +1163,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mahagi</t>
+          <t>Lubero</t>
         </is>
       </c>
       <c r="B23">
-        <v>0.06174990321331785</v>
+        <v>0.07028165576731223</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1169,10 +1175,10 @@
         </is>
       </c>
       <c r="D23">
-        <v>0.6713187694549561</v>
+        <v>0.7601358294487</v>
       </c>
       <c r="E23">
-        <v>2.717971801757812E-05</v>
+        <v>9.5367431640625E-07</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1183,7 +1189,7 @@
         <v>4</v>
       </c>
       <c r="H23">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1194,11 +1200,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ariwara</t>
+          <t>Aungba</t>
         </is>
       </c>
       <c r="B24">
-        <v>0.07160493827160494</v>
+        <v>0.07999666332999666</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1206,10 +1212,10 @@
         </is>
       </c>
       <c r="D24">
-        <v>0.6630400419235229</v>
+        <v>0.693227231502533</v>
       </c>
       <c r="E24">
-        <v>3.302097320556641E-05</v>
+        <v>5.602836608886719E-06</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1220,7 +1226,7 @@
         <v>4</v>
       </c>
       <c r="H24">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1235,7 +1241,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>0.07351055809390281</v>
+        <v>0.08964597582483762</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1243,10 +1249,10 @@
         </is>
       </c>
       <c r="D25">
-        <v>0.713412880897522</v>
+        <v>0.7143549919128418</v>
       </c>
       <c r="E25">
-        <v>7.390975952148438E-06</v>
+        <v>3.337860107421875E-06</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1257,7 +1263,7 @@
         <v>4</v>
       </c>
       <c r="H25">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1268,11 +1274,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Drodro</t>
+          <t>Rimba</t>
         </is>
       </c>
       <c r="B26">
-        <v>0.07478632478632478</v>
+        <v>0.0898172594088109</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1280,10 +1286,10 @@
         </is>
       </c>
       <c r="D26">
-        <v>0.694214403629303</v>
+        <v>0.423763245344162</v>
       </c>
       <c r="E26">
-        <v>9.655952453613281E-06</v>
+        <v>0.00685584545135498</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1294,7 +1300,7 @@
         <v>4</v>
       </c>
       <c r="H26">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1305,11 +1311,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Buta</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="B27">
-        <v>0.07515746124031007</v>
+        <v>0.09126180836707153</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1317,10 +1323,10 @@
         </is>
       </c>
       <c r="D27">
-        <v>0.5487046241760254</v>
+        <v>0.6904374957084656</v>
       </c>
       <c r="E27">
-        <v>0.00136256217956543</v>
+        <v>5.960464477539062E-06</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1331,7 +1337,7 @@
         <v>4</v>
       </c>
       <c r="H27">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1342,11 +1348,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pawa</t>
+          <t>Boma Mangbetu</t>
         </is>
       </c>
       <c r="B28">
-        <v>0.08273495971407578</v>
+        <v>0.09144837952407492</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1354,10 +1360,10 @@
         </is>
       </c>
       <c r="D28">
-        <v>0.697837233543396</v>
+        <v>0.6621222496032715</v>
       </c>
       <c r="E28">
-        <v>1.502037048339844E-05</v>
+        <v>3.230571746826172E-05</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1365,10 +1371,10 @@
         </is>
       </c>
       <c r="G28">
-        <v>3.666666666666667</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="H28">
-        <v>0.3865079365079365</v>
+        <v>0.2194444444444444</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1379,11 +1385,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mabalako</t>
+          <t>Mahagi</t>
         </is>
       </c>
       <c r="B29">
-        <v>0.08997682998343517</v>
+        <v>0.09601238869531553</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1391,10 +1397,10 @@
         </is>
       </c>
       <c r="D29">
-        <v>0.7570013403892517</v>
+        <v>0.6667926907539368</v>
       </c>
       <c r="E29">
-        <v>1.549720764160156E-06</v>
+        <v>1.835823059082031E-05</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1405,7 +1411,7 @@
         <v>4</v>
       </c>
       <c r="H29">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1416,11 +1422,11 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Buta</t>
         </is>
       </c>
       <c r="B30">
-        <v>0.09143049932523617</v>
+        <v>0.1037427325581395</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1428,10 +1434,10 @@
         </is>
       </c>
       <c r="D30">
-        <v>0.7302387952804565</v>
+        <v>0.6075541973114014</v>
       </c>
       <c r="E30">
-        <v>3.099441528320312E-06</v>
+        <v>0.0002446174621582031</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1442,7 +1448,7 @@
         <v>4</v>
       </c>
       <c r="H30">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1453,11 +1459,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Boma Mangbetu</t>
+          <t>Musienene</t>
         </is>
       </c>
       <c r="B31">
-        <v>0.0924693050685088</v>
+        <v>0.1509246467876047</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1465,10 +1471,10 @@
         </is>
       </c>
       <c r="D31">
-        <v>0.6101983785629272</v>
+        <v>0.4525650143623352</v>
       </c>
       <c r="E31">
-        <v>0.0002561807632446289</v>
+        <v>0.002658486366271973</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1476,10 +1482,10 @@
         </is>
       </c>
       <c r="G31">
-        <v>2.666666666666667</v>
+        <v>2.833333333333333</v>
       </c>
       <c r="H31">
-        <v>0.4462121212121212</v>
+        <v>0.4941077441077441</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1490,11 +1496,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Aungba</t>
+          <t>Wamba</t>
         </is>
       </c>
       <c r="B32">
-        <v>0.1039372706039373</v>
+        <v>0.1642486864240349</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1502,10 +1508,10 @@
         </is>
       </c>
       <c r="D32">
-        <v>0.6822270154953003</v>
+        <v>0.7273017168045044</v>
       </c>
       <c r="E32">
-        <v>1.740455627441406E-05</v>
+        <v>4.529953002929688E-06</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1513,10 +1519,10 @@
         </is>
       </c>
       <c r="G32">
-        <v>4</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="H32">
-        <v>0.3049138104028578</v>
+        <v>0.2101449275362319</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1527,11 +1533,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Musienene</t>
+          <t>Pawa</t>
         </is>
       </c>
       <c r="B33">
-        <v>0.1198355983833437</v>
+        <v>0.1664300149963971</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1539,10 +1545,10 @@
         </is>
       </c>
       <c r="D33">
-        <v>0.4571774303913116</v>
+        <v>0.7908952236175537</v>
       </c>
       <c r="E33">
-        <v>0.003279805183410645</v>
+        <v>4.76837158203125E-07</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1550,10 +1556,10 @@
         </is>
       </c>
       <c r="G33">
-        <v>4.333333333333333</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="H33">
-        <v>0.342483660130719</v>
+        <v>0.3747061406907954</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1564,11 +1570,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Oicha</t>
+          <t>Mabalako</t>
         </is>
       </c>
       <c r="B34">
-        <v>0.1222680769006141</v>
+        <v>0.1829205777601597</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1576,10 +1582,10 @@
         </is>
       </c>
       <c r="D34">
-        <v>0.6104573011398315</v>
+        <v>0.7356088757514954</v>
       </c>
       <c r="E34">
-        <v>9.787082672119141E-05</v>
+        <v>1.192092895507812E-06</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1587,10 +1593,10 @@
         </is>
       </c>
       <c r="G34">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="H34">
-        <v>0.3049138104028578</v>
+        <v>0.275494755710583</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1601,11 +1607,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Beni</t>
+          <t>Isiro</t>
         </is>
       </c>
       <c r="B35">
-        <v>0.1366258753905095</v>
+        <v>0.1938552977473861</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1613,10 +1619,10 @@
         </is>
       </c>
       <c r="D35">
-        <v>0.3447233140468597</v>
+        <v>0.7494383454322815</v>
       </c>
       <c r="E35">
-        <v>0.02429091930389404</v>
+        <v>1.311302185058594E-06</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1624,10 +1630,10 @@
         </is>
       </c>
       <c r="G35">
-        <v>4.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="H35">
-        <v>0.3373913668031315</v>
+        <v>0.2118660472319009</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1638,11 +1644,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Wamba</t>
+          <t>Damas</t>
         </is>
       </c>
       <c r="B36">
-        <v>0.1561598712005745</v>
+        <v>0.2224470296492015</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1650,10 +1656,10 @@
         </is>
       </c>
       <c r="D36">
-        <v>0.7719165086746216</v>
+        <v>0.794860303401947</v>
       </c>
       <c r="E36">
-        <v>2.026557922363281E-06</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1661,10 +1667,10 @@
         </is>
       </c>
       <c r="G36">
-        <v>5</v>
+        <v>6.333333333333333</v>
       </c>
       <c r="H36">
-        <v>0.1588874928257868</v>
+        <v>0.06060606060606061</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1679,7 +1685,7 @@
         </is>
       </c>
       <c r="B37">
-        <v>0.2074512133525836</v>
+        <v>0.225450979705092</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1687,7 +1693,7 @@
         </is>
       </c>
       <c r="D37">
-        <v>0.8041196465492249</v>
+        <v>0.7774868607521057</v>
       </c>
       <c r="E37">
         <v>3.576278686523438E-07</v>
@@ -1698,10 +1704,10 @@
         </is>
       </c>
       <c r="G37">
-        <v>4.333333333333333</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="H37">
-        <v>0.3370035265769863</v>
+        <v>0.4122388324396503</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -1712,11 +1718,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Damas</t>
+          <t>Vuhovi</t>
         </is>
       </c>
       <c r="B38">
-        <v>0.2129504661699751</v>
+        <v>0.2573944050199758</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1724,10 +1730,10 @@
         </is>
       </c>
       <c r="D38">
-        <v>0.7482962608337402</v>
+        <v>0.6423118114471436</v>
       </c>
       <c r="E38">
-        <v>2.86102294921875E-06</v>
+        <v>2.837181091308594E-05</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1735,10 +1741,10 @@
         </is>
       </c>
       <c r="G38">
-        <v>8.333333333333334</v>
+        <v>4</v>
       </c>
       <c r="H38">
-        <v>0.09794628751974724</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1749,11 +1755,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Isiro</t>
+          <t>Beni</t>
         </is>
       </c>
       <c r="B39">
-        <v>0.2396142007755405</v>
+        <v>0.2642756852322419</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1761,10 +1767,10 @@
         </is>
       </c>
       <c r="D39">
-        <v>0.7898502945899963</v>
+        <v>0.3663225173950195</v>
       </c>
       <c r="E39">
-        <v>8.344650268554688E-07</v>
+        <v>0.01380836963653564</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1772,10 +1778,10 @@
         </is>
       </c>
       <c r="G39">
-        <v>4.666666666666667</v>
+        <v>6.333333333333333</v>
       </c>
       <c r="H39">
-        <v>0.1884097384097384</v>
+        <v>0.2759477124183006</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -1786,11 +1792,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Mandima</t>
+          <t>Bambu</t>
         </is>
       </c>
       <c r="B40">
-        <v>0.239755265420159</v>
+        <v>0.2912291401815624</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1798,10 +1804,10 @@
         </is>
       </c>
       <c r="D40">
-        <v>0.8077446222305298</v>
+        <v>0.6520128846168518</v>
       </c>
       <c r="E40">
-        <v>2.384185791015625E-07</v>
+        <v>1.263618469238281E-05</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1809,10 +1815,10 @@
         </is>
       </c>
       <c r="G40">
-        <v>2.5</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="H40">
-        <v>0.5079365079365079</v>
+        <v>0.3518356643356643</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -1823,11 +1829,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bambu</t>
+          <t>Oicha</t>
         </is>
       </c>
       <c r="B41">
-        <v>0.2731801997977928</v>
+        <v>0.3112655820017649</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1835,10 +1841,10 @@
         </is>
       </c>
       <c r="D41">
-        <v>0.7274523973464966</v>
+        <v>0.7045202851295471</v>
       </c>
       <c r="E41">
-        <v>1.9073486328125E-06</v>
+        <v>2.86102294921875E-06</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1846,10 +1852,10 @@
         </is>
       </c>
       <c r="G41">
-        <v>4.833333333333333</v>
+        <v>4</v>
       </c>
       <c r="H41">
-        <v>0.3432098765432098</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -1864,7 +1870,7 @@
         </is>
       </c>
       <c r="B42">
-        <v>0.2815088194454701</v>
+        <v>0.3122381253882437</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1872,7 +1878,7 @@
         </is>
       </c>
       <c r="D42">
-        <v>0.8531813025474548</v>
+        <v>0.8529959917068481</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -1891,11 +1897,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Katwa</t>
+          <t>Mandima</t>
         </is>
       </c>
       <c r="B43">
-        <v>0.312387434382387</v>
+        <v>0.3172595076614314</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1903,10 +1909,10 @@
         </is>
       </c>
       <c r="D43">
-        <v>0.786450207233429</v>
+        <v>0.770475447177887</v>
       </c>
       <c r="E43">
-        <v>2.384185791015625E-07</v>
+        <v>3.576278686523438E-07</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1914,25 +1920,25 @@
         </is>
       </c>
       <c r="G43">
-        <v>1.666666666666667</v>
+        <v>5.333333333333333</v>
       </c>
       <c r="H43">
-        <v>0.483704137392662</v>
+        <v>0.3166666666666667</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Under-alerting &amp; Rapid</t>
+          <t>Under-alerting &amp; Delayed</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mambasa</t>
+          <t>Katwa</t>
         </is>
       </c>
       <c r="B44">
-        <v>0.3270803270803271</v>
+        <v>0.3274197472707039</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1940,10 +1946,10 @@
         </is>
       </c>
       <c r="D44">
-        <v>0.6026270389556885</v>
+        <v>0.8372437953948975</v>
       </c>
       <c r="E44">
-        <v>0.0001060962677001953</v>
+        <v>0</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1951,10 +1957,10 @@
         </is>
       </c>
       <c r="G44">
-        <v>4</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="H44">
-        <v>0.3049138104028578</v>
+        <v>0.3196471394313121</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -1965,11 +1971,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Lolwa</t>
+          <t>Nia Nia</t>
         </is>
       </c>
       <c r="B45">
-        <v>0.3287864336251433</v>
+        <v>0.3338961427051504</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1977,10 +1983,10 @@
         </is>
       </c>
       <c r="D45">
-        <v>0.826751708984375</v>
+        <v>0.7071495056152344</v>
       </c>
       <c r="E45">
-        <v>1.192092895507812E-07</v>
+        <v>3.814697265625E-06</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1988,10 +1994,10 @@
         </is>
       </c>
       <c r="G45">
-        <v>3.666666666666667</v>
+        <v>3</v>
       </c>
       <c r="H45">
-        <v>0.2601398601398601</v>
+        <v>0.4448661184904069</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2002,11 +2008,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Vuhovi</t>
+          <t>Lolwa</t>
         </is>
       </c>
       <c r="B46">
-        <v>0.3331506849315068</v>
+        <v>0.3459669919977447</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -2014,10 +2020,10 @@
         </is>
       </c>
       <c r="D46">
-        <v>0.6474369168281555</v>
+        <v>0.782903254032135</v>
       </c>
       <c r="E46">
-        <v>4.160404205322266E-05</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2028,7 +2034,7 @@
         <v>4</v>
       </c>
       <c r="H46">
-        <v>0.3049138104028578</v>
+        <v>0.1881313131313131</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2043,7 +2049,7 @@
         </is>
       </c>
       <c r="B47">
-        <v>0.3496628253302178</v>
+        <v>0.3576026557377741</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -2051,10 +2057,10 @@
         </is>
       </c>
       <c r="D47">
-        <v>0.7915222644805908</v>
+        <v>0.7922484278678894</v>
       </c>
       <c r="E47">
-        <v>2.384185791015625E-07</v>
+        <v>1.192092895507812E-07</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2062,10 +2068,10 @@
         </is>
       </c>
       <c r="G47">
-        <v>3.166666666666667</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="H47">
-        <v>0.4421526789947843</v>
+        <v>0.3240454076367389</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -2076,11 +2082,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Kyondo</t>
+          <t>Aru</t>
         </is>
       </c>
       <c r="B48">
-        <v>0.3576734629366208</v>
+        <v>0.3621247369004099</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -2088,10 +2094,10 @@
         </is>
       </c>
       <c r="D48">
-        <v>0.7872794270515442</v>
+        <v>0.5076889395713806</v>
       </c>
       <c r="E48">
-        <v>4.76837158203125E-07</v>
+        <v>0.0007269382476806641</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2102,7 +2108,7 @@
         <v>4</v>
       </c>
       <c r="H48">
-        <v>0.3049138104028578</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2113,11 +2119,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Nia Nia</t>
+          <t>Mongbwalu</t>
         </is>
       </c>
       <c r="B49">
-        <v>0.3846241698679564</v>
+        <v>0.4100982250271306</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -2125,10 +2131,10 @@
         </is>
       </c>
       <c r="D49">
-        <v>0.77248215675354</v>
+        <v>0.3660646080970764</v>
       </c>
       <c r="E49">
-        <v>8.344650268554688E-07</v>
+        <v>0.0145193338394165</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2136,10 +2142,10 @@
         </is>
       </c>
       <c r="G49">
-        <v>2.666666666666667</v>
+        <v>5.166666666666667</v>
       </c>
       <c r="H49">
-        <v>0.4295958802478834</v>
+        <v>0.273668041070418</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2150,11 +2156,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Lita</t>
+          <t>Kyondo</t>
         </is>
       </c>
       <c r="B50">
-        <v>0.4054594991803289</v>
+        <v>0.4457819821523893</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -2162,10 +2168,10 @@
         </is>
       </c>
       <c r="D50">
-        <v>0.6715693473815918</v>
+        <v>0.8366318941116333</v>
       </c>
       <c r="E50">
-        <v>1.537799835205078E-05</v>
+        <v>0</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2173,10 +2179,10 @@
         </is>
       </c>
       <c r="G50">
-        <v>4.166666666666667</v>
+        <v>4</v>
       </c>
       <c r="H50">
-        <v>0.3241335044929397</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2187,11 +2193,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Aru</t>
+          <t>Rwampara</t>
         </is>
       </c>
       <c r="B51">
-        <v>0.413135593220339</v>
+        <v>0.4646199198069724</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2199,10 +2205,10 @@
         </is>
       </c>
       <c r="D51">
-        <v>0.5104763507843018</v>
+        <v>0.5374996662139893</v>
       </c>
       <c r="E51">
-        <v>0.0009365081787109375</v>
+        <v>0.0002858638763427734</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2210,10 +2216,10 @@
         </is>
       </c>
       <c r="G51">
-        <v>4</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="H51">
-        <v>0.3049138104028578</v>
+        <v>0.212985532985533</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2224,11 +2230,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mongbwalu</t>
+          <t>Nizi</t>
         </is>
       </c>
       <c r="B52">
-        <v>0.4347646343051526</v>
+        <v>0.4708222786758258</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -2236,10 +2242,10 @@
         </is>
       </c>
       <c r="D52">
-        <v>0.3879620134830475</v>
+        <v>0.7488955855369568</v>
       </c>
       <c r="E52">
-        <v>0.01212871074676514</v>
+        <v>5.960464477539062E-07</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2247,10 +2253,10 @@
         </is>
       </c>
       <c r="G52">
-        <v>4.5</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="H52">
-        <v>0.3579309860144775</v>
+        <v>0.3055555555555556</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2261,11 +2267,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Kilo</t>
+          <t>Lita</t>
         </is>
       </c>
       <c r="B53">
-        <v>0.4566773504273504</v>
+        <v>0.4943555217858623</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -2273,10 +2279,10 @@
         </is>
       </c>
       <c r="D53">
-        <v>0.6162175536155701</v>
+        <v>0.7116370797157288</v>
       </c>
       <c r="E53">
-        <v>7.832050323486328E-05</v>
+        <v>2.026557922363281E-06</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2284,10 +2290,10 @@
         </is>
       </c>
       <c r="G53">
-        <v>4</v>
+        <v>4.166666666666667</v>
       </c>
       <c r="H53">
-        <v>0.3049138104028578</v>
+        <v>0.3819689254471863</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -2298,11 +2304,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Rwampara</t>
+          <t>Mangala</t>
         </is>
       </c>
       <c r="B54">
-        <v>0.4698832252985488</v>
+        <v>0.5014038946386558</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -2310,10 +2316,10 @@
         </is>
       </c>
       <c r="D54">
-        <v>0.6494230628013611</v>
+        <v>0.7742227911949158</v>
       </c>
       <c r="E54">
-        <v>1.823902130126953E-05</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2321,10 +2327,10 @@
         </is>
       </c>
       <c r="G54">
-        <v>4.333333333333333</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="H54">
-        <v>0.194563320176789</v>
+        <v>0.2131896268147428</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -2335,11 +2341,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Nizi</t>
+          <t>Bunia</t>
         </is>
       </c>
       <c r="B55">
-        <v>0.5610050156750866</v>
+        <v>0.5330369188714826</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -2347,10 +2353,10 @@
         </is>
       </c>
       <c r="D55">
-        <v>0.7661417126655579</v>
+        <v>0.5321540236473083</v>
       </c>
       <c r="E55">
-        <v>5.960464477539062E-07</v>
+        <v>0.0003403425216674805</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2358,10 +2364,10 @@
         </is>
       </c>
       <c r="G55">
-        <v>4.666666666666667</v>
+        <v>4</v>
       </c>
       <c r="H55">
-        <v>0.2250037086485684</v>
+        <v>0.3587355089117001</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -2372,11 +2378,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Bunia</t>
+          <t>Kilo</t>
         </is>
       </c>
       <c r="B56">
-        <v>0.5632497755485184</v>
+        <v>0.56875</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2384,10 +2390,10 @@
         </is>
       </c>
       <c r="D56">
-        <v>0.6360458135604858</v>
+        <v>0.5594550371170044</v>
       </c>
       <c r="E56">
-        <v>2.849102020263672E-05</v>
+        <v>0.0002081394195556641</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2398,7 +2404,7 @@
         <v>4</v>
       </c>
       <c r="H56">
-        <v>0.3349204748645349</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -2409,11 +2415,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Mangala</t>
+          <t>Mambasa</t>
         </is>
       </c>
       <c r="B57">
-        <v>0.59461501633818</v>
+        <v>0.6125541125541125</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2421,10 +2427,10 @@
         </is>
       </c>
       <c r="D57">
-        <v>0.8172613382339478</v>
+        <v>0.6970254182815552</v>
       </c>
       <c r="E57">
-        <v>1.192092895507812E-07</v>
+        <v>3.576278686523438E-06</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2432,10 +2438,10 @@
         </is>
       </c>
       <c r="G57">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="H57">
-        <v>0.1532452859591709</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -2450,7 +2456,7 @@
         </is>
       </c>
       <c r="B58">
-        <v>0.8957624894400564</v>
+        <v>0.8888423611653518</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -2458,10 +2464,10 @@
         </is>
       </c>
       <c r="D58">
-        <v>0.5454531311988831</v>
+        <v>0.5631020069122314</v>
       </c>
       <c r="E58">
-        <v>0.0004222393035888672</v>
+        <v>0.000165104866027832</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2469,10 +2475,10 @@
         </is>
       </c>
       <c r="G58">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="H58">
-        <v>0.4914648060382658</v>
+        <v>0.3980410375532327</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -2487,7 +2493,7 @@
         </is>
       </c>
       <c r="B59">
-        <v>1.340476190476191</v>
+        <v>1.259523809523809</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -2495,10 +2501,10 @@
         </is>
       </c>
       <c r="D59">
-        <v>0.7735267877578735</v>
+        <v>0.8094488382339478</v>
       </c>
       <c r="E59">
-        <v>5.960464477539062E-07</v>
+        <v>1.192092895507812E-07</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -2509,7 +2515,7 @@
         <v>4</v>
       </c>
       <c r="H59">
-        <v>0.244610296025861</v>
+        <v>0.3051578305744758</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: refresh ShinyApp artifacts after threshold spike fix
Refreshed 01/01b thresholds and trend outputs to reflect the
degenerate-week exclusion fix (commit 17d3021). Wamba and Boma
Mangbetu Sep windows now show smooth decay (53->41->22, 14->19->0)
instead of the 9x spike seen in the previous run.

Vuhovi (34x jump at 2026-09-06) remains a sparse-data issue
requiring cross-zone Bayesian shrinkage - out of scope.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ShinyApp/data/02_recent_adequacy.xlsx
+++ b/ShinyApp/data/02_recent_adequacy.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -416,10 +416,10 @@
         </is>
       </c>
       <c r="D2">
-        <v>-0.2165144085884094</v>
+        <v>-0.2190890163183212</v>
       </c>
       <c r="E2">
-        <v>0.2228713780641556</v>
+        <v>0.1972127556800842</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -447,10 +447,10 @@
         </is>
       </c>
       <c r="D3">
-        <v>-0.04624922573566437</v>
+        <v>-0.03651483729481697</v>
       </c>
       <c r="E3">
-        <v>0.8169167041778564</v>
+        <v>0.8538416028022766</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -478,21 +478,15 @@
         </is>
       </c>
       <c r="D4">
-        <v>0.210282951593399</v>
+        <v>0.1963452994823456</v>
       </c>
       <c r="E4">
-        <v>0.1997592449188232</v>
+        <v>0.222248911857605</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
-      </c>
-      <c r="G4">
-        <v>4</v>
-      </c>
-      <c r="H4">
-        <v>0.3037569944044764</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -515,10 +509,10 @@
         </is>
       </c>
       <c r="D5">
-        <v>-0.1292644441127777</v>
+        <v>-0.1179383844137192</v>
       </c>
       <c r="E5">
-        <v>0.4387663602828979</v>
+        <v>0.4780884087085724</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -546,21 +540,15 @@
         </is>
       </c>
       <c r="D6">
-        <v>0.2177862077951431</v>
+        <v>0.1872764229774475</v>
       </c>
       <c r="E6">
-        <v>0.2296985387802124</v>
+        <v>0.2929122447967529</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>Stable</t>
         </is>
-      </c>
-      <c r="G6">
-        <v>4</v>
-      </c>
-      <c r="H6">
-        <v>0.3037569944044764</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -571,11 +559,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gombari</t>
+          <t>Ganga</t>
         </is>
       </c>
       <c r="B7">
-        <v>0.004761904761904762</v>
+        <v>0.00392156862745098</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -583,10 +571,10 @@
         </is>
       </c>
       <c r="D7">
-        <v>0.4658205211162567</v>
+        <v>0.3640728294849396</v>
       </c>
       <c r="E7">
-        <v>0.00719749927520752</v>
+        <v>0.03338158130645752</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -597,7 +585,7 @@
         <v>4</v>
       </c>
       <c r="H7">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -608,11 +596,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tshopo</t>
+          <t>Adja</t>
         </is>
       </c>
       <c r="B8">
-        <v>0.008620689655172414</v>
+        <v>0.003968253968253968</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -620,10 +608,10 @@
         </is>
       </c>
       <c r="D8">
-        <v>0.4841409027576447</v>
+        <v>0.3685627281665802</v>
       </c>
       <c r="E8">
-        <v>0.004570364952087402</v>
+        <v>0.02311420440673828</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -634,7 +622,7 @@
         <v>4</v>
       </c>
       <c r="H8">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -645,11 +633,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Mangobo</t>
+          <t>Basali</t>
         </is>
       </c>
       <c r="B9">
-        <v>0.009878193701723114</v>
+        <v>0.005747126436781609</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -657,21 +645,21 @@
         </is>
       </c>
       <c r="D9">
-        <v>0.4092455208301544</v>
+        <v>0.1563471853733063</v>
       </c>
       <c r="E9">
-        <v>0.01411116123199463</v>
+        <v>0.3799142837524414</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Increasing</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="G9">
         <v>4</v>
       </c>
       <c r="H9">
-        <v>0.3051578305744758</v>
+        <v>0.2872983870967742</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -682,11 +670,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Makiso Kisangani</t>
+          <t>Wanierukula</t>
         </is>
       </c>
       <c r="B10">
-        <v>0.01383838383838384</v>
+        <v>0.01388888888888889</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -694,10 +682,10 @@
         </is>
       </c>
       <c r="D10">
-        <v>0.57316654920578</v>
+        <v>0.403007984161377</v>
       </c>
       <c r="E10">
-        <v>0.0003368854522705078</v>
+        <v>0.01569092273712158</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -708,7 +696,7 @@
         <v>4</v>
       </c>
       <c r="H10">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -719,11 +707,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kabondo</t>
+          <t>Gombari</t>
         </is>
       </c>
       <c r="B11">
-        <v>0.01572327044025157</v>
+        <v>0.01428571428571429</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -731,10 +719,10 @@
         </is>
       </c>
       <c r="D11">
-        <v>0.5474497079849243</v>
+        <v>0.5645250678062439</v>
       </c>
       <c r="E11">
-        <v>0.000800013542175293</v>
+        <v>0.0007451772689819336</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -745,7 +733,7 @@
         <v>4</v>
       </c>
       <c r="H11">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -756,11 +744,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Ganga</t>
+          <t>Mangobo</t>
         </is>
       </c>
       <c r="B12">
-        <v>0.01631393298059965</v>
+        <v>0.02235862272358623</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -768,10 +756,10 @@
         </is>
       </c>
       <c r="D12">
-        <v>0.4845437407493591</v>
+        <v>0.5135525465011597</v>
       </c>
       <c r="E12">
-        <v>0.005962848663330078</v>
+        <v>0.001497745513916016</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -782,7 +770,7 @@
         <v>4</v>
       </c>
       <c r="H12">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -793,11 +781,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Butembo</t>
+          <t>Rungu</t>
         </is>
       </c>
       <c r="B13">
-        <v>0.01783216783216783</v>
+        <v>0.02740740740740741</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -805,21 +793,21 @@
         </is>
       </c>
       <c r="D13">
-        <v>0.008116412907838821</v>
+        <v>0.5518492460250854</v>
       </c>
       <c r="E13">
-        <v>0.9793041944503784</v>
+        <v>0.0007729530334472656</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Stable</t>
+          <t>Increasing</t>
         </is>
       </c>
       <c r="G13">
         <v>4</v>
       </c>
       <c r="H13">
-        <v>0.3058582486594755</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -830,11 +818,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Wanierukula</t>
+          <t>Tshopo</t>
         </is>
       </c>
       <c r="B14">
-        <v>0.02083333333333334</v>
+        <v>0.02817034105897871</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -842,10 +830,10 @@
         </is>
       </c>
       <c r="D14">
-        <v>0.3696977496147156</v>
+        <v>0.6338549256324768</v>
       </c>
       <c r="E14">
-        <v>0.02988338470458984</v>
+        <v>9.787082672119141E-05</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -856,7 +844,7 @@
         <v>4</v>
       </c>
       <c r="H14">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -867,11 +855,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Adja</t>
+          <t>Makiso Kisangani</t>
         </is>
       </c>
       <c r="B15">
-        <v>0.02380952380952381</v>
+        <v>0.03271424620848253</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -879,10 +867,10 @@
         </is>
       </c>
       <c r="D15">
-        <v>0.4639152884483337</v>
+        <v>0.7762150764465332</v>
       </c>
       <c r="E15">
-        <v>0.004813671112060547</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -890,10 +878,10 @@
         </is>
       </c>
       <c r="G15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H15">
-        <v>0.3051578305744758</v>
+        <v>0.5111111111111111</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -904,11 +892,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kambala</t>
+          <t>Dungu</t>
         </is>
       </c>
       <c r="B16">
-        <v>0.02718052738336714</v>
+        <v>0.03409961685823755</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -916,10 +904,10 @@
         </is>
       </c>
       <c r="D16">
-        <v>0.390964537858963</v>
+        <v>0.4712323248386383</v>
       </c>
       <c r="E16">
-        <v>0.01713776588439941</v>
+        <v>0.00507819652557373</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -930,7 +918,7 @@
         <v>4</v>
       </c>
       <c r="H16">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -941,11 +929,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rungu</t>
+          <t>Kambala</t>
         </is>
       </c>
       <c r="B17">
-        <v>0.02740740740740741</v>
+        <v>0.03475321162947938</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -953,10 +941,10 @@
         </is>
       </c>
       <c r="D17">
-        <v>0.6635317802429199</v>
+        <v>0.4262419939041138</v>
       </c>
       <c r="E17">
-        <v>6.771087646484375E-05</v>
+        <v>0.007238864898681641</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -967,7 +955,7 @@
         <v>4</v>
       </c>
       <c r="H17">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -978,11 +966,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Drodro</t>
+          <t>Kabondo</t>
         </is>
       </c>
       <c r="B18">
-        <v>0.03472222222222222</v>
+        <v>0.0406857015639784</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -990,10 +978,10 @@
         </is>
       </c>
       <c r="D18">
-        <v>0.5603131055831909</v>
+        <v>0.5960424542427063</v>
       </c>
       <c r="E18">
-        <v>0.0002535581588745117</v>
+        <v>0.0001701116561889648</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1004,7 +992,7 @@
         <v>4</v>
       </c>
       <c r="H18">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1027,10 +1015,10 @@
         </is>
       </c>
       <c r="D19">
-        <v>0.7224345207214355</v>
+        <v>0.7504051327705383</v>
       </c>
       <c r="E19">
-        <v>7.748603820800781E-06</v>
+        <v>2.145767211914062E-06</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1041,7 +1029,7 @@
         <v>4</v>
       </c>
       <c r="H19">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1052,11 +1040,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ariwara</t>
+          <t>Drodro</t>
         </is>
       </c>
       <c r="B20">
-        <v>0.04444444444444445</v>
+        <v>0.0486111111111111</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1064,10 +1052,10 @@
         </is>
       </c>
       <c r="D20">
-        <v>0.562595546245575</v>
+        <v>0.5688654780387878</v>
       </c>
       <c r="E20">
-        <v>0.0003312826156616211</v>
+        <v>0.000147700309753418</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1078,7 +1066,7 @@
         <v>4</v>
       </c>
       <c r="H20">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1093,7 +1081,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>0.04547803617571059</v>
+        <v>0.05322997416020672</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1101,10 +1089,10 @@
         </is>
       </c>
       <c r="D21">
-        <v>0.3697565793991089</v>
+        <v>0.4511842727661133</v>
       </c>
       <c r="E21">
-        <v>0.02267980575561523</v>
+        <v>0.004046201705932617</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1115,7 +1103,7 @@
         <v>4</v>
       </c>
       <c r="H21">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1126,11 +1114,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Bafwasende</t>
+          <t>Aungba</t>
         </is>
       </c>
       <c r="B22">
-        <v>0.05450636394908841</v>
+        <v>0.05839172505839172</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1138,10 +1126,10 @@
         </is>
       </c>
       <c r="D22">
-        <v>0.5139064788818359</v>
+        <v>0.6490340828895569</v>
       </c>
       <c r="E22">
-        <v>0.001737356185913086</v>
+        <v>1.442432403564453E-05</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1152,7 +1140,7 @@
         <v>4</v>
       </c>
       <c r="H22">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1167,7 +1155,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>0.07028165576731223</v>
+        <v>0.05888132808773645</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1175,10 +1163,10 @@
         </is>
       </c>
       <c r="D23">
-        <v>0.7601358294487</v>
+        <v>0.7835034728050232</v>
       </c>
       <c r="E23">
-        <v>9.5367431640625E-07</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1189,7 +1177,7 @@
         <v>4</v>
       </c>
       <c r="H23">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1200,11 +1188,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Aungba</t>
+          <t>Ariwara</t>
         </is>
       </c>
       <c r="B24">
-        <v>0.07999666332999666</v>
+        <v>0.0617283950617284</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1212,10 +1200,10 @@
         </is>
       </c>
       <c r="D24">
-        <v>0.693227231502533</v>
+        <v>0.6280551552772522</v>
       </c>
       <c r="E24">
-        <v>5.602836608886719E-06</v>
+        <v>3.409385681152344E-05</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1226,7 +1214,7 @@
         <v>4</v>
       </c>
       <c r="H24">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1237,11 +1225,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Gety</t>
+          <t>Vuhovi</t>
         </is>
       </c>
       <c r="B25">
-        <v>0.08964597582483762</v>
+        <v>0.06969507101086048</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1249,10 +1237,10 @@
         </is>
       </c>
       <c r="D25">
-        <v>0.7143549919128418</v>
+        <v>0.5429861545562744</v>
       </c>
       <c r="E25">
-        <v>3.337860107421875E-06</v>
+        <v>0.0003371238708496094</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1263,7 +1251,7 @@
         <v>4</v>
       </c>
       <c r="H25">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1274,11 +1262,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Rimba</t>
+          <t>Butembo</t>
         </is>
       </c>
       <c r="B26">
-        <v>0.0898172594088109</v>
+        <v>0.07645687645687646</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1286,21 +1274,21 @@
         </is>
       </c>
       <c r="D26">
-        <v>0.423763245344162</v>
+        <v>0.1679682433605194</v>
       </c>
       <c r="E26">
-        <v>0.00685584545135498</v>
+        <v>0.2754685878753662</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Increasing</t>
+          <t>Stable</t>
         </is>
       </c>
       <c r="G26">
         <v>4</v>
       </c>
       <c r="H26">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1311,11 +1299,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Logo</t>
+          <t>Gety</t>
         </is>
       </c>
       <c r="B27">
-        <v>0.09126180836707153</v>
+        <v>0.08640817177402543</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1323,10 +1311,10 @@
         </is>
       </c>
       <c r="D27">
-        <v>0.6904374957084656</v>
+        <v>0.7754946947097778</v>
       </c>
       <c r="E27">
-        <v>5.960464477539062E-06</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1337,7 +1325,7 @@
         <v>4</v>
       </c>
       <c r="H27">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -1348,11 +1336,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Boma Mangbetu</t>
+          <t>Rimba</t>
         </is>
       </c>
       <c r="B28">
-        <v>0.09144837952407492</v>
+        <v>0.09245742092457421</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1360,10 +1348,10 @@
         </is>
       </c>
       <c r="D28">
-        <v>0.6621222496032715</v>
+        <v>0.4880935251712799</v>
       </c>
       <c r="E28">
-        <v>3.230571746826172E-05</v>
+        <v>0.001371979713439941</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1371,10 +1359,10 @@
         </is>
       </c>
       <c r="G28">
-        <v>4.166666666666667</v>
+        <v>4</v>
       </c>
       <c r="H28">
-        <v>0.2194444444444444</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1385,11 +1373,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mahagi</t>
+          <t>Logo</t>
         </is>
       </c>
       <c r="B29">
-        <v>0.09601238869531553</v>
+        <v>0.1002024291497976</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1397,10 +1385,10 @@
         </is>
       </c>
       <c r="D29">
-        <v>0.6667926907539368</v>
+        <v>0.7137183547019958</v>
       </c>
       <c r="E29">
-        <v>1.835823059082031E-05</v>
+        <v>1.430511474609375E-06</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1411,7 +1399,7 @@
         <v>4</v>
       </c>
       <c r="H29">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1426,7 +1414,7 @@
         </is>
       </c>
       <c r="B30">
-        <v>0.1037427325581395</v>
+        <v>0.1039244186046512</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1434,10 +1422,10 @@
         </is>
       </c>
       <c r="D30">
-        <v>0.6075541973114014</v>
+        <v>0.6285796761512756</v>
       </c>
       <c r="E30">
-        <v>0.0002446174621582031</v>
+        <v>9.071826934814453E-05</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1448,7 +1436,7 @@
         <v>4</v>
       </c>
       <c r="H30">
-        <v>0.3051578305744758</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -1459,11 +1447,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Musienene</t>
+          <t>Mahagi</t>
         </is>
       </c>
       <c r="B31">
-        <v>0.1509246467876047</v>
+        <v>0.1066589237320945</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1471,10 +1459,10 @@
         </is>
       </c>
       <c r="D31">
-        <v>0.4525650143623352</v>
+        <v>0.6932860612869263</v>
       </c>
       <c r="E31">
-        <v>0.002658486366271973</v>
+        <v>4.887580871582031E-06</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1482,10 +1470,10 @@
         </is>
       </c>
       <c r="G31">
-        <v>2.833333333333333</v>
+        <v>4</v>
       </c>
       <c r="H31">
-        <v>0.4941077441077441</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -1496,11 +1484,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Wamba</t>
+          <t>Boma Mangbetu</t>
         </is>
       </c>
       <c r="B32">
-        <v>0.1642486864240349</v>
+        <v>0.1148580121703854</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1508,10 +1496,10 @@
         </is>
       </c>
       <c r="D32">
-        <v>0.7273017168045044</v>
+        <v>0.6701478958129883</v>
       </c>
       <c r="E32">
-        <v>4.529953002929688E-06</v>
+        <v>1.788139343261719E-05</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1519,10 +1507,10 @@
         </is>
       </c>
       <c r="G32">
-        <v>4.666666666666667</v>
+        <v>4.333333333333333</v>
       </c>
       <c r="H32">
-        <v>0.2101449275362319</v>
+        <v>0.2096560846560847</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -1533,11 +1521,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pawa</t>
+          <t>Bafwasende</t>
         </is>
       </c>
       <c r="B33">
-        <v>0.1664300149963971</v>
+        <v>0.1240299823633157</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1545,10 +1533,10 @@
         </is>
       </c>
       <c r="D33">
-        <v>0.7908952236175537</v>
+        <v>0.6757950782775879</v>
       </c>
       <c r="E33">
-        <v>4.76837158203125E-07</v>
+        <v>2.074241638183594E-05</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1556,10 +1544,10 @@
         </is>
       </c>
       <c r="G33">
-        <v>3.666666666666667</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="H33">
-        <v>0.3747061406907954</v>
+        <v>0.365993265993266</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -1570,11 +1558,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mabalako</t>
+          <t>Musienene</t>
         </is>
       </c>
       <c r="B34">
-        <v>0.1829205777601597</v>
+        <v>0.136181360919394</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1582,10 +1570,10 @@
         </is>
       </c>
       <c r="D34">
-        <v>0.7356088757514954</v>
+        <v>0.4925181269645691</v>
       </c>
       <c r="E34">
-        <v>1.192092895507812E-06</v>
+        <v>0.0008178949356079102</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1593,10 +1581,10 @@
         </is>
       </c>
       <c r="G34">
-        <v>5.5</v>
+        <v>2.666666666666667</v>
       </c>
       <c r="H34">
-        <v>0.275494755710583</v>
+        <v>0.4958464958464958</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -1607,11 +1595,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Isiro</t>
+          <t>Mabalako</t>
         </is>
       </c>
       <c r="B35">
-        <v>0.1938552977473861</v>
+        <v>0.1655888460252521</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1619,10 +1607,10 @@
         </is>
       </c>
       <c r="D35">
-        <v>0.7494383454322815</v>
+        <v>0.7525984048843384</v>
       </c>
       <c r="E35">
-        <v>1.311302185058594E-06</v>
+        <v>4.76837158203125E-07</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1630,10 +1618,10 @@
         </is>
       </c>
       <c r="G35">
-        <v>4</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="H35">
-        <v>0.2118660472319009</v>
+        <v>0.2767857142857143</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
@@ -1644,11 +1632,11 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Damas</t>
+          <t>Wamba</t>
         </is>
       </c>
       <c r="B36">
-        <v>0.2224470296492015</v>
+        <v>0.1681985980638368</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1656,10 +1644,10 @@
         </is>
       </c>
       <c r="D36">
-        <v>0.794860303401947</v>
+        <v>0.7407437562942505</v>
       </c>
       <c r="E36">
-        <v>2.384185791015625E-07</v>
+        <v>1.430511474609375E-06</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1667,10 +1655,10 @@
         </is>
       </c>
       <c r="G36">
-        <v>6.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="H36">
-        <v>0.06060606060606061</v>
+        <v>0.3251082251082251</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -1681,11 +1669,11 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Fataki</t>
+          <t>Damas</t>
         </is>
       </c>
       <c r="B37">
-        <v>0.225450979705092</v>
+        <v>0.1748254281949934</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1693,10 +1681,10 @@
         </is>
       </c>
       <c r="D37">
-        <v>0.7774868607521057</v>
+        <v>0.7397730350494385</v>
       </c>
       <c r="E37">
-        <v>3.576278686523438E-07</v>
+        <v>9.5367431640625E-07</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1704,10 +1692,10 @@
         </is>
       </c>
       <c r="G37">
-        <v>3.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="H37">
-        <v>0.4122388324396503</v>
+        <v>0.2265993265993266</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
@@ -1718,11 +1706,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Vuhovi</t>
+          <t>Isiro</t>
         </is>
       </c>
       <c r="B38">
-        <v>0.2573944050199758</v>
+        <v>0.1839583396242891</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1730,10 +1718,10 @@
         </is>
       </c>
       <c r="D38">
-        <v>0.6423118114471436</v>
+        <v>0.7397730350494385</v>
       </c>
       <c r="E38">
-        <v>2.837181091308594E-05</v>
+        <v>9.5367431640625E-07</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1744,7 +1732,7 @@
         <v>4</v>
       </c>
       <c r="H38">
-        <v>0.3051578305744758</v>
+        <v>0.2303544494720965</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -1755,11 +1743,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Beni</t>
+          <t>Fataki</t>
         </is>
       </c>
       <c r="B39">
-        <v>0.2642756852322419</v>
+        <v>0.1865088995595002</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1767,10 +1755,10 @@
         </is>
       </c>
       <c r="D39">
-        <v>0.3663225173950195</v>
+        <v>0.7313984632492065</v>
       </c>
       <c r="E39">
-        <v>0.01380836963653564</v>
+        <v>9.5367431640625E-07</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1778,10 +1766,10 @@
         </is>
       </c>
       <c r="G39">
-        <v>6.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="H39">
-        <v>0.2759477124183006</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -1792,11 +1780,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bambu</t>
+          <t>Pawa</t>
         </is>
       </c>
       <c r="B40">
-        <v>0.2912291401815624</v>
+        <v>0.208789199800278</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1804,10 +1792,10 @@
         </is>
       </c>
       <c r="D40">
-        <v>0.6520128846168518</v>
+        <v>0.7826237082481384</v>
       </c>
       <c r="E40">
-        <v>1.263618469238281E-05</v>
+        <v>2.384185791015625E-07</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1815,10 +1803,10 @@
         </is>
       </c>
       <c r="G40">
-        <v>4.666666666666667</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="H40">
-        <v>0.3518356643356643</v>
+        <v>0.3986678986678986</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -1829,11 +1817,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Oicha</t>
+          <t>Ensemble de la zone affectée</t>
         </is>
       </c>
       <c r="B41">
-        <v>0.3112655820017649</v>
+        <v>0.3030408716475391</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1841,21 +1829,15 @@
         </is>
       </c>
       <c r="D41">
-        <v>0.7045202851295471</v>
+        <v>0.8313867449760437</v>
       </c>
       <c r="E41">
-        <v>2.86102294921875E-06</v>
+        <v>0</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>Increasing</t>
         </is>
-      </c>
-      <c r="G41">
-        <v>4</v>
-      </c>
-      <c r="H41">
-        <v>0.3051578305744758</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -1866,11 +1848,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Ensemble de la zone affectée</t>
+          <t>Bambu</t>
         </is>
       </c>
       <c r="B42">
-        <v>0.3122381253882437</v>
+        <v>0.3059880989188257</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1878,15 +1860,21 @@
         </is>
       </c>
       <c r="D42">
-        <v>0.8529959917068481</v>
+        <v>0.6350852847099304</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>1.275539398193359E-05</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>Increasing</t>
         </is>
+      </c>
+      <c r="G42">
+        <v>3.833333333333333</v>
+      </c>
+      <c r="H42">
+        <v>0.3946986201888162</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
@@ -1897,11 +1885,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mandima</t>
+          <t>Beni</t>
         </is>
       </c>
       <c r="B43">
-        <v>0.3172595076614314</v>
+        <v>0.3100030505462001</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1909,10 +1897,10 @@
         </is>
       </c>
       <c r="D43">
-        <v>0.770475447177887</v>
+        <v>0.4095229506492615</v>
       </c>
       <c r="E43">
-        <v>3.576278686523438E-07</v>
+        <v>0.004930257797241211</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1920,10 +1908,10 @@
         </is>
       </c>
       <c r="G43">
-        <v>5.333333333333333</v>
+        <v>6.333333333333333</v>
       </c>
       <c r="H43">
-        <v>0.3166666666666667</v>
+        <v>0.2280287844653764</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -1934,11 +1922,11 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Katwa</t>
+          <t>Komanda</t>
         </is>
       </c>
       <c r="B44">
-        <v>0.3274197472707039</v>
+        <v>0.3492733940899073</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1946,7 +1934,7 @@
         </is>
       </c>
       <c r="D44">
-        <v>0.8372437953948975</v>
+        <v>0.811201810836792</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -1957,10 +1945,10 @@
         </is>
       </c>
       <c r="G44">
-        <v>3.666666666666667</v>
+        <v>5</v>
       </c>
       <c r="H44">
-        <v>0.3196471394313121</v>
+        <v>0.3021298609533903</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -1971,11 +1959,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Nia Nia</t>
+          <t>Lolwa</t>
         </is>
       </c>
       <c r="B45">
-        <v>0.3338961427051504</v>
+        <v>0.3702942668696093</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1983,10 +1971,10 @@
         </is>
       </c>
       <c r="D45">
-        <v>0.7071495056152344</v>
+        <v>0.7394348382949829</v>
       </c>
       <c r="E45">
-        <v>3.814697265625E-06</v>
+        <v>5.960464477539062E-07</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1994,10 +1982,10 @@
         </is>
       </c>
       <c r="G45">
-        <v>3</v>
+        <v>3.833333333333333</v>
       </c>
       <c r="H45">
-        <v>0.4448661184904069</v>
+        <v>0.2148148148148148</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2008,11 +1996,11 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Lolwa</t>
+          <t>Katwa</t>
         </is>
       </c>
       <c r="B46">
-        <v>0.3459669919977447</v>
+        <v>0.4092815288947161</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -2020,10 +2008,10 @@
         </is>
       </c>
       <c r="D46">
-        <v>0.782903254032135</v>
+        <v>0.857601523399353</v>
       </c>
       <c r="E46">
-        <v>2.384185791015625E-07</v>
+        <v>0</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -2031,10 +2019,10 @@
         </is>
       </c>
       <c r="G46">
-        <v>4</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="H46">
-        <v>0.1881313131313131</v>
+        <v>0.2889256750264607</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2045,11 +2033,11 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Komanda</t>
+          <t>Aru</t>
         </is>
       </c>
       <c r="B47">
-        <v>0.3576026557377741</v>
+        <v>0.4244350282485875</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -2057,10 +2045,10 @@
         </is>
       </c>
       <c r="D47">
-        <v>0.7922484278678894</v>
+        <v>0.5674931406974792</v>
       </c>
       <c r="E47">
-        <v>1.192092895507812E-07</v>
+        <v>0.000125885009765625</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -2068,10 +2056,10 @@
         </is>
       </c>
       <c r="G47">
-        <v>4.333333333333333</v>
+        <v>4</v>
       </c>
       <c r="H47">
-        <v>0.3240454076367389</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
@@ -2082,11 +2070,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Aru</t>
+          <t>Lita</t>
         </is>
       </c>
       <c r="B48">
-        <v>0.3621247369004099</v>
+        <v>0.4246396930586316</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -2094,10 +2082,10 @@
         </is>
       </c>
       <c r="D48">
-        <v>0.5076889395713806</v>
+        <v>0.6880975961685181</v>
       </c>
       <c r="E48">
-        <v>0.0007269382476806641</v>
+        <v>3.099441528320312E-06</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2105,10 +2093,10 @@
         </is>
       </c>
       <c r="G48">
-        <v>4</v>
+        <v>3.666666666666667</v>
       </c>
       <c r="H48">
-        <v>0.3051578305744758</v>
+        <v>0.4093118094642485</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
@@ -2119,11 +2107,11 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mongbwalu</t>
+          <t>Oicha</t>
         </is>
       </c>
       <c r="B49">
-        <v>0.4100982250271306</v>
+        <v>0.4270870050145983</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -2131,10 +2119,10 @@
         </is>
       </c>
       <c r="D49">
-        <v>0.3660646080970764</v>
+        <v>0.7298004627227783</v>
       </c>
       <c r="E49">
-        <v>0.0145193338394165</v>
+        <v>7.152557373046875E-07</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2142,10 +2130,10 @@
         </is>
       </c>
       <c r="G49">
-        <v>5.166666666666667</v>
+        <v>4</v>
       </c>
       <c r="H49">
-        <v>0.273668041070418</v>
+        <v>0.2575122292103424</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
@@ -2156,11 +2144,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Kyondo</t>
+          <t>Nia Nia</t>
         </is>
       </c>
       <c r="B50">
-        <v>0.4457819821523893</v>
+        <v>0.4337018143434452</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -2168,10 +2156,10 @@
         </is>
       </c>
       <c r="D50">
-        <v>0.8366318941116333</v>
+        <v>0.7276438474655151</v>
       </c>
       <c r="E50">
-        <v>0</v>
+        <v>1.072883605957031E-06</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2179,10 +2167,10 @@
         </is>
       </c>
       <c r="G50">
-        <v>4</v>
+        <v>3.333333333333333</v>
       </c>
       <c r="H50">
-        <v>0.3051578305744758</v>
+        <v>0.3899389590918826</v>
       </c>
       <c r="I50" t="inlineStr">
         <is>
@@ -2193,11 +2181,11 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rwampara</t>
+          <t>Mangala</t>
         </is>
       </c>
       <c r="B51">
-        <v>0.4646199198069724</v>
+        <v>0.4352482011480314</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -2205,10 +2193,10 @@
         </is>
       </c>
       <c r="D51">
-        <v>0.5374996662139893</v>
+        <v>0.7923548221588135</v>
       </c>
       <c r="E51">
-        <v>0.0002858638763427734</v>
+        <v>1.192092895507812E-07</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2216,10 +2204,10 @@
         </is>
       </c>
       <c r="G51">
-        <v>4.666666666666667</v>
+        <v>5.666666666666667</v>
       </c>
       <c r="H51">
-        <v>0.212985532985533</v>
+        <v>0.2284522642212985</v>
       </c>
       <c r="I51" t="inlineStr">
         <is>
@@ -2230,11 +2218,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nizi</t>
+          <t>Mongbwalu</t>
         </is>
       </c>
       <c r="B52">
-        <v>0.4708222786758258</v>
+        <v>0.4533237954021026</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -2242,10 +2230,10 @@
         </is>
       </c>
       <c r="D52">
-        <v>0.7488955855369568</v>
+        <v>0.387814998626709</v>
       </c>
       <c r="E52">
-        <v>5.960464477539062E-07</v>
+        <v>0.008347868919372559</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2253,10 +2241,10 @@
         </is>
       </c>
       <c r="G52">
-        <v>4.166666666666667</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="H52">
-        <v>0.3055555555555556</v>
+        <v>0.2393065998329156</v>
       </c>
       <c r="I52" t="inlineStr">
         <is>
@@ -2267,11 +2255,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Lita</t>
+          <t>Kyondo</t>
         </is>
       </c>
       <c r="B53">
-        <v>0.4943555217858623</v>
+        <v>0.463998867288341</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -2279,10 +2267,10 @@
         </is>
       </c>
       <c r="D53">
-        <v>0.7116370797157288</v>
+        <v>0.8592524528503418</v>
       </c>
       <c r="E53">
-        <v>2.026557922363281E-06</v>
+        <v>0</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2290,10 +2278,10 @@
         </is>
       </c>
       <c r="G53">
-        <v>4.166666666666667</v>
+        <v>4</v>
       </c>
       <c r="H53">
-        <v>0.3819689254471863</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I53" t="inlineStr">
         <is>
@@ -2304,11 +2292,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mangala</t>
+          <t>Mambasa</t>
         </is>
       </c>
       <c r="B54">
-        <v>0.5014038946386558</v>
+        <v>0.4670701726257281</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -2316,10 +2304,10 @@
         </is>
       </c>
       <c r="D54">
-        <v>0.7742227911949158</v>
+        <v>0.6878445744514465</v>
       </c>
       <c r="E54">
-        <v>2.384185791015625E-07</v>
+        <v>2.980232238769531E-06</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2327,10 +2315,10 @@
         </is>
       </c>
       <c r="G54">
-        <v>5.666666666666667</v>
+        <v>4</v>
       </c>
       <c r="H54">
-        <v>0.2131896268147428</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I54" t="inlineStr">
         <is>
@@ -2341,11 +2329,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bunia</t>
+          <t>Kilo</t>
         </is>
       </c>
       <c r="B55">
-        <v>0.5330369188714826</v>
+        <v>0.46720947063689</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -2353,10 +2341,10 @@
         </is>
       </c>
       <c r="D55">
-        <v>0.5321540236473083</v>
+        <v>0.5461092591285706</v>
       </c>
       <c r="E55">
-        <v>0.0003403425216674805</v>
+        <v>0.0002402067184448242</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2367,7 +2355,7 @@
         <v>4</v>
       </c>
       <c r="H55">
-        <v>0.3587355089117001</v>
+        <v>0.2977228026870449</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -2378,11 +2366,11 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Kilo</t>
+          <t>Nizi</t>
         </is>
       </c>
       <c r="B56">
-        <v>0.56875</v>
+        <v>0.474816155771797</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -2390,10 +2378,10 @@
         </is>
       </c>
       <c r="D56">
-        <v>0.5594550371170044</v>
+        <v>0.707925021648407</v>
       </c>
       <c r="E56">
-        <v>0.0002081394195556641</v>
+        <v>1.192092895507812E-06</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2404,7 +2392,7 @@
         <v>4</v>
       </c>
       <c r="H56">
-        <v>0.3051578305744758</v>
+        <v>0.3032561198082389</v>
       </c>
       <c r="I56" t="inlineStr">
         <is>
@@ -2415,11 +2403,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Mambasa</t>
+          <t>Rwampara</t>
         </is>
       </c>
       <c r="B57">
-        <v>0.6125541125541125</v>
+        <v>0.4758985017205389</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -2427,10 +2415,10 @@
         </is>
       </c>
       <c r="D57">
-        <v>0.6970254182815552</v>
+        <v>0.5795717835426331</v>
       </c>
       <c r="E57">
-        <v>3.576278686523438E-06</v>
+        <v>5.793571472167969E-05</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2438,10 +2426,10 @@
         </is>
       </c>
       <c r="G57">
-        <v>4</v>
+        <v>4.666666666666667</v>
       </c>
       <c r="H57">
-        <v>0.3051578305744758</v>
+        <v>0.2197548523324324</v>
       </c>
       <c r="I57" t="inlineStr">
         <is>
@@ -2452,22 +2440,22 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Nyankunde</t>
+          <t>Mandima</t>
         </is>
       </c>
       <c r="B58">
-        <v>0.8888423611653518</v>
+        <v>0.5316121276592852</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Adequate</t>
+          <t>Under-alerting</t>
         </is>
       </c>
       <c r="D58">
-        <v>0.5631020069122314</v>
+        <v>0.8776472210884094</v>
       </c>
       <c r="E58">
-        <v>0.000165104866027832</v>
+        <v>0</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2475,49 +2463,123 @@
         </is>
       </c>
       <c r="G58">
-        <v>4.5</v>
+        <v>6.666666666666667</v>
       </c>
       <c r="H58">
-        <v>0.3980410375532327</v>
+        <v>0.2767676767676768</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>Adequate Volume &amp; Delayed</t>
+          <t>Under-alerting &amp; Delayed</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>Bunia</t>
+        </is>
+      </c>
+      <c r="B59">
+        <v>0.5370035323177249</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Under-alerting</t>
+        </is>
+      </c>
+      <c r="D59">
+        <v>0.5135603547096252</v>
+      </c>
+      <c r="E59">
+        <v>0.0004048347473144531</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Increasing</t>
+        </is>
+      </c>
+      <c r="G59">
+        <v>4</v>
+      </c>
+      <c r="H59">
+        <v>0.3279941926005208</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Under-alerting &amp; Delayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
           <t>Tchomia</t>
         </is>
       </c>
-      <c r="B59">
-        <v>1.259523809523809</v>
-      </c>
-      <c r="C59" t="inlineStr">
+      <c r="B60">
+        <v>1.159920634920635</v>
+      </c>
+      <c r="C60" t="inlineStr">
         <is>
           <t>Adequate</t>
         </is>
       </c>
-      <c r="D59">
-        <v>0.8094488382339478</v>
-      </c>
-      <c r="E59">
-        <v>1.192092895507812E-07</v>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Increasing</t>
-        </is>
-      </c>
-      <c r="G59">
-        <v>4</v>
-      </c>
-      <c r="H59">
-        <v>0.3051578305744758</v>
-      </c>
-      <c r="I59" t="inlineStr">
+      <c r="D60">
+        <v>0.8062557578086853</v>
+      </c>
+      <c r="E60">
+        <v>0</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Increasing</t>
+        </is>
+      </c>
+      <c r="G60">
+        <v>4</v>
+      </c>
+      <c r="H60">
+        <v>0.2650628700271123</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Adequate Volume &amp; Delayed</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Nyankunde</t>
+        </is>
+      </c>
+      <c r="B61">
+        <v>1.179423416225573</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Adequate</t>
+        </is>
+      </c>
+      <c r="D61">
+        <v>0.6098179817199707</v>
+      </c>
+      <c r="E61">
+        <v>3.087520599365234E-05</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Increasing</t>
+        </is>
+      </c>
+      <c r="G61">
+        <v>7</v>
+      </c>
+      <c r="H61">
+        <v>0.2920634920634921</v>
+      </c>
+      <c r="I61" t="inlineStr">
         <is>
           <t>Adequate Volume &amp; Delayed</t>
         </is>

</xml_diff>